<commit_message>
Modify first year, week one, day one
</commit_message>
<xml_diff>
--- a/Planificación de clases.xlsx
+++ b/Planificación de clases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="5"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Primer año" sheetId="1" state="visible" r:id="rId1"/>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">Modulo 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Distribuciones de Linux - ¿Qué es Linux? y preparación de herramientas (Rufus + ISO Fedora)</t>
+    <t xml:space="preserve">Distribuciones de Linux · Preparación de Herramientas · Ventoy + ISO Windows + ISO Fedora</t>
   </si>
   <si>
     <t xml:space="preserve">Flashear ISO de Fedora en USB con Rufus desde Windows, Boot Live y configuración de BIOS/UEFI</t>
@@ -652,8 +652,8 @@
       <top style="thin">
         <color theme="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -671,9 +671,9 @@
       <right style="thin">
         <color theme="1"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -693,11 +693,11 @@
       <right style="thin">
         <color theme="1"/>
       </right>
-      <top/>
+      <top style="none"/>
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="none"/>

</xml_diff>